<commit_message>
Final sync: Generated JSON correlation rules and removed redundant manual Sigma updates
</commit_message>
<xml_diff>
--- a/techniques_table.xlsx
+++ b/techniques_table.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Covered Techniques" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Uncovered Techniques" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -123,34 +134,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CoveredTechniquesTable" displayName="CoveredTechniquesTable" ref="A1:F128" headerRowCount="1">
-  <autoFilter ref="A1:F128"/>
-  <tableColumns count="6">
-    <tableColumn id="1" name="Parent ID"/>
-    <tableColumn id="2" name="Technique Name"/>
-    <tableColumn id="3" name="Tactics"/>
-    <tableColumn id="4" name="Subtechniques Covered"/>
-    <tableColumn id="5" name="Rules Count"/>
-    <tableColumn id="6" name="Rule Sources"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="UncoveredTechniquesTable" displayName="UncoveredTechniquesTable" ref="A1:D63" headerRowCount="1">
-  <autoFilter ref="A1:D63"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Parent ID"/>
-    <tableColumn id="2" name="Technique Name"/>
-    <tableColumn id="3" name="Tactics"/>
-    <tableColumn id="4" name="Platform"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -444,42 +427,34 @@
   </sheetPr>
   <dimension ref="A1:F195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="49" customWidth="1" min="2" max="2"/>
-    <col width="61" customWidth="1" min="3" max="3"/>
-    <col width="63" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Parent ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Technique Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Tactics</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Subtechniques Covered</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Rules Count</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Rule Sources</t>
         </is>
@@ -3709,7 +3684,7 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -3739,7 +3714,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -4546,6 +4521,8 @@
       <c r="D137" t="n">
         <v>1</v>
       </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4566,6 +4543,8 @@
       <c r="D138" t="n">
         <v>1</v>
       </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4586,6 +4565,8 @@
       <c r="D139" t="n">
         <v>1</v>
       </c>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4606,6 +4587,8 @@
       <c r="D140" t="n">
         <v>1</v>
       </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -4626,6 +4609,8 @@
       <c r="D141" t="n">
         <v>1</v>
       </c>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -4646,6 +4631,8 @@
       <c r="D142" t="n">
         <v>1</v>
       </c>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -6345,53 +6332,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Parent ID</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Technique Name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Tactics</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Platform</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>